<commit_message>
Update latest FINE electronic finance data
</commit_message>
<xml_diff>
--- a/전자금융업_최신.xlsx
+++ b/전자금융업_최신.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FSS_15U50Q\Desktop\★2026 전금감\2. 전금업 등록업무\1. 등록 및 말소 현황\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBDA310-E43B-4A5B-BC06-83E10C091C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D16A38-D25F-4A0F-9094-23ABBBE9DADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="813" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="813" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="전자금융업 등록 현황" sheetId="2" r:id="rId1"/>
@@ -1123,7 +1123,8 @@
             <family val="3"/>
             <charset val="129"/>
           </rPr>
-          <t>(구) 원페이</t>
+          <t>(구) 원페이
+(구) 위드페이먼츠</t>
         </r>
       </text>
     </comment>
@@ -4961,7 +4962,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="681">
   <si>
     <t>업 체 명</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -7787,6 +7788,18 @@
   <si>
     <t>케이아이에스정보통신 주식회사</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>주식회사 세프라</t>
+  </si>
+  <si>
+    <t>주식회사 치우천소프트</t>
+  </si>
+  <si>
+    <t>640-87-03320</t>
+  </si>
+  <si>
+    <t>884-87-03143</t>
   </si>
 </sst>
 </file>
@@ -8092,7 +8105,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -8283,6 +8296,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -8781,8 +8797,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표33" displayName="표33" ref="B5:K247" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="B5:K247" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표33" displayName="표33" ref="B5:K249" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="B5:K249" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No." dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="등록날짜" dataDxfId="8"/>
@@ -9160,7 +9176,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K253"/>
+  <dimension ref="A1:K255"/>
   <sheetFormatPr defaultColWidth="20.6640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="19" customWidth="1"/>
@@ -9200,7 +9216,7 @@
     </row>
     <row r="3" spans="2:11" ht="13.5" x14ac:dyDescent="0.15">
       <c r="I3" s="56">
-        <v>46260</v>
+        <v>46315</v>
       </c>
       <c r="J3" s="56"/>
     </row>
@@ -14911,62 +14927,88 @@
     </row>
     <row r="247" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A247" s="29"/>
-      <c r="B247" s="27"/>
-      <c r="C247" s="21" t="s">
+      <c r="B247" s="64">
+        <v>242</v>
+      </c>
+      <c r="C247" s="33">
+        <v>46315</v>
+      </c>
+      <c r="D247" s="15" t="s">
+        <v>677</v>
+      </c>
+      <c r="E247" s="53" t="s">
+        <v>679</v>
+      </c>
+      <c r="F247" s="36"/>
+      <c r="G247" s="36"/>
+      <c r="H247" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="I247" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="J247" s="36"/>
+      <c r="K247" s="36"/>
+    </row>
+    <row r="248" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A248" s="29"/>
+      <c r="B248" s="64">
+        <v>243</v>
+      </c>
+      <c r="C248" s="33">
+        <v>46315</v>
+      </c>
+      <c r="D248" s="15" t="s">
+        <v>678</v>
+      </c>
+      <c r="E248" s="53" t="s">
+        <v>680</v>
+      </c>
+      <c r="F248" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="G248" s="36"/>
+      <c r="H248" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="I248" s="36"/>
+      <c r="J248" s="36"/>
+      <c r="K248" s="36"/>
+    </row>
+    <row r="249" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B249" s="27"/>
+      <c r="C249" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D247" s="41" t="str">
-        <f>CONCATENATE("총 ",COUNTA($D6:$D246),"개사"," (",SUM($F247:$K247),"개 업종)")</f>
-        <v>총 241개사 (407개 업종)</v>
-      </c>
-      <c r="E247" s="51"/>
-      <c r="F247" s="22">
-        <f>COUNTA(F6:F246)</f>
-        <v>119</v>
-      </c>
-      <c r="G247" s="22">
-        <f>COUNTA(G6:G246)</f>
+      <c r="D249" s="41" t="str">
+        <f>CONCATENATE("총 ",COUNTA($D6:$D248),"개사"," (",SUM($F249:$K249),"개 업종)")</f>
+        <v>총 243개사 (411개 업종)</v>
+      </c>
+      <c r="E249" s="51"/>
+      <c r="F249" s="22">
+        <f>COUNTA(F6:F248)</f>
+        <v>120</v>
+      </c>
+      <c r="G249" s="22">
+        <f t="shared" ref="G249:J249" si="0">COUNTA(G6:G248)</f>
         <v>35</v>
       </c>
-      <c r="H247" s="22">
-        <f>COUNTA(H6:H246)</f>
-        <v>190</v>
-      </c>
-      <c r="I247" s="22">
-        <f>COUNTA(I6:I246)</f>
-        <v>45</v>
-      </c>
-      <c r="J247" s="22">
-        <f>COUNTA(J6:J246)</f>
+      <c r="H249" s="22">
+        <f t="shared" si="0"/>
+        <v>192</v>
+      </c>
+      <c r="I249" s="22">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="J249" s="22">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="K247" s="39">
+      <c r="K249" s="39">
         <f>COUNTA(K6:K144)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="248" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A248" s="29"/>
-      <c r="B248" s="30"/>
-      <c r="C248" s="31"/>
-      <c r="D248" s="31"/>
-      <c r="E248" s="31"/>
-      <c r="F248" s="31"/>
-      <c r="G248" s="31"/>
-      <c r="H248" s="31"/>
-      <c r="I248" s="31"/>
-      <c r="J248" s="31"/>
-    </row>
-    <row r="249" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B249" s="30"/>
-      <c r="C249" s="31"/>
-      <c r="D249" s="31"/>
-      <c r="E249" s="31"/>
-      <c r="F249" s="31"/>
-      <c r="G249" s="31"/>
-      <c r="H249" s="31"/>
-      <c r="I249" s="31"/>
-      <c r="J249" s="31"/>
     </row>
     <row r="250" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B250" s="30"/>
@@ -14982,7 +15024,9 @@
     <row r="251" spans="1:11" x14ac:dyDescent="0.15">
       <c r="B251" s="30"/>
       <c r="C251" s="31"/>
-      <c r="F251" s="52"/>
+      <c r="D251" s="31"/>
+      <c r="E251" s="31"/>
+      <c r="F251" s="31"/>
       <c r="G251" s="31"/>
       <c r="H251" s="31"/>
       <c r="I251" s="31"/>
@@ -15002,13 +15046,33 @@
     <row r="253" spans="1:11" x14ac:dyDescent="0.15">
       <c r="B253" s="30"/>
       <c r="C253" s="31"/>
-      <c r="D253" s="31"/>
-      <c r="E253" s="31"/>
-      <c r="F253" s="31"/>
+      <c r="F253" s="52"/>
       <c r="G253" s="31"/>
       <c r="H253" s="31"/>
       <c r="I253" s="31"/>
       <c r="J253" s="31"/>
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="B254" s="30"/>
+      <c r="C254" s="31"/>
+      <c r="D254" s="31"/>
+      <c r="E254" s="31"/>
+      <c r="F254" s="31"/>
+      <c r="G254" s="31"/>
+      <c r="H254" s="31"/>
+      <c r="I254" s="31"/>
+      <c r="J254" s="31"/>
+    </row>
+    <row r="255" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="B255" s="30"/>
+      <c r="C255" s="31"/>
+      <c r="D255" s="31"/>
+      <c r="E255" s="31"/>
+      <c r="F255" s="31"/>
+      <c r="G255" s="31"/>
+      <c r="H255" s="31"/>
+      <c r="I255" s="31"/>
+      <c r="J255" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>